<commit_message>
tweaking for AA deficits
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_25_07_02.xlsx
+++ b/simulations/scene/inputs/Scenarios_25_07_02.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp15056\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\root_cynaps\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D83380-7B9A-4D02-BA87-129AD2650F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D37933-2356-46C4-BF68-4E8B74C52B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1447,7 +1447,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1485,7 +1485,6 @@
     <xf numFmtId="0" fontId="18" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="11" fontId="16" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="11" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1970,54 +1969,54 @@
       <c r="G3" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="H3" s="22">
+      <c r="H3" s="21">
         <v>1.0000000000000001E-9</v>
       </c>
-      <c r="I3" s="23">
+      <c r="I3" s="22">
         <f>6.417000259344E-08/3600</f>
         <v>1.78250007204E-11</v>
       </c>
-      <c r="J3" s="23">
+      <c r="J3" s="22">
         <f>4.504500274824E-08/3600</f>
         <v>1.2512500763399999E-11</v>
       </c>
-      <c r="K3" s="23">
+      <c r="K3" s="22">
         <f>6.26400201772801E-08/3600</f>
         <v>1.7400005604800025E-11</v>
       </c>
-      <c r="L3" s="23">
+      <c r="L3" s="22">
         <f>0.0000001715700135192/3600</f>
         <v>4.7658337088666669E-11</v>
       </c>
-      <c r="M3" s="23">
+      <c r="M3" s="22">
         <f>0.0000005947500532344/3600</f>
         <v>1.6520834812066667E-10</v>
       </c>
-      <c r="N3" s="23">
+      <c r="N3" s="22">
         <f>0.0000014904001011456/3600</f>
         <v>4.1400002809600001E-10</v>
       </c>
-      <c r="O3" s="23">
+      <c r="O3" s="22">
         <f>0.000002756700138744/3600</f>
         <v>7.6575003854E-10</v>
       </c>
-      <c r="P3" s="23">
+      <c r="P3" s="22">
         <f>0.00000411600012288/3600</f>
         <v>1.1433333674666667E-9</v>
       </c>
-      <c r="Q3" s="23">
+      <c r="Q3" s="22">
         <f>0.000004950000112896/3600</f>
         <v>1.3750000313600002E-9</v>
       </c>
-      <c r="R3" s="23">
+      <c r="R3" s="22">
         <f>5.14350001490399E-06/3600</f>
         <v>1.4287500041399972E-9</v>
       </c>
-      <c r="S3" s="23">
+      <c r="S3" s="22">
         <f>4.82699998247999E-06/3600</f>
         <v>1.3408333284666637E-9</v>
       </c>
-      <c r="T3" s="23">
+      <c r="T3" s="22">
         <f>4.18949994376799E-06/3600</f>
         <v>1.1637499843799972E-9</v>
       </c>
@@ -2146,7 +2145,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>237</v>
       </c>
@@ -2169,59 +2168,59 @@
         <v>0.5</v>
       </c>
       <c r="H6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" ref="H6:T6" si="0">0.00005 / 100</f>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="I6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="J6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="K6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="L6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="M6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="N6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="O6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="P6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="Q6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="R6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="S6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="T6" s="10">
-        <f>0.00005 / 100</f>
+        <f t="shared" si="0"/>
         <v>4.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>240</v>
       </c>
@@ -2283,7 +2282,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="8" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>243</v>
       </c>
@@ -2306,59 +2305,59 @@
         <v>0.5</v>
       </c>
       <c r="H8" s="10">
-        <f t="shared" ref="H8:T8" si="0">0.00002 / 14</f>
+        <f t="shared" ref="H8:T8" si="1">0.00002 / 14</f>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="I8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="J8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="K8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="L8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="M8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="N8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="O8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="P8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="Q8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="R8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="S8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
       <c r="T8" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4285714285714286E-6</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>194</v>
       </c>
@@ -2420,7 +2419,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>195</v>
       </c>
@@ -2482,7 +2481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>196</v>
       </c>
@@ -2568,55 +2567,55 @@
         <v>1.2499999999999999E-6</v>
       </c>
       <c r="H12" s="20">
-        <f t="shared" ref="H12:T12" si="1">1250*0.000001/5</f>
+        <f t="shared" ref="H12:T12" si="2">1250*0.000001/5</f>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="I12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="J12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="K12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="L12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="M12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="N12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="O12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="P12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="Q12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="R12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="S12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="T12" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5000000000000001E-4</v>
       </c>
     </row>
@@ -2705,55 +2704,55 @@
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="H14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" ref="H14:T14" si="3" xml:space="preserve"> 0.0000000000025*10</f>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="I14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="J14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="K14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="L14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="M14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="N14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="O14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="P14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="Q14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="R14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="S14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
       <c r="T14" s="10">
-        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <f t="shared" si="3"/>
         <v>2.4999999999999998E-11</v>
       </c>
     </row>
@@ -2780,48 +2779,48 @@
         <v>1.2E-8</v>
       </c>
       <c r="H15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" ref="H15:R15" si="4">0.00000000005 *2</f>
         <v>1E-10</v>
       </c>
       <c r="I15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="J15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="K15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="L15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="M15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="N15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="O15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="P15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="Q15" s="10">
-        <f>0.00000000005 *2</f>
+        <f t="shared" si="4"/>
         <v>1E-10</v>
       </c>
       <c r="R15" s="10">
-        <f>0.00000000001 / 10</f>
-        <v>9.9999999999999998E-13</v>
+        <f>0.00000000005 / 5 / 10</f>
+        <v>1.0000000000000002E-12</v>
       </c>
       <c r="S15" s="10">
         <f>0.00000000005 *2</f>
@@ -2992,55 +2991,55 @@
         <v>9.9999999999999995E-8</v>
       </c>
       <c r="H18" s="10">
-        <f t="shared" ref="H18:T18" si="2">0.000001 / 10000 / 4 / 10</f>
+        <f t="shared" ref="H18:T18" si="5">0.000001 / 10000 / 4 / 10</f>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="I18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="J18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="K18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="L18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="M18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="N18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="O18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="P18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="Q18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="R18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="S18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="T18" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.4999999999999998E-12</v>
       </c>
     </row>
@@ -3068,55 +3067,55 @@
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="H19" s="10">
-        <f t="shared" ref="H19:T19" si="3">0.00001</f>
+        <f t="shared" ref="H19:T19" si="6">0.00001</f>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="I19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="J19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="K19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="L19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="M19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="N19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="O19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="P19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="Q19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="R19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="S19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="T19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
@@ -3144,55 +3143,55 @@
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="H20" s="10">
-        <f t="shared" ref="H20:T20" si="4" xml:space="preserve"> 0.001 * 10</f>
+        <f t="shared" ref="H20:T20" si="7" xml:space="preserve"> 0.001 * 10</f>
         <v>0.01</v>
       </c>
       <c r="I20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="J20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="K20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="L20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="M20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="N20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="O20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="P20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="Q20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="R20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="S20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
       <c r="T20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.01</v>
       </c>
     </row>
@@ -3219,55 +3218,55 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="H21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" ref="H21:T21" si="8">0.00001 / 10 / 2 / 4</f>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="I21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="J21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="K21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="L21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="M21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="N21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="O21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="P21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="Q21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="R21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="S21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
       <c r="T21" s="10">
-        <f>0.00001 / 10 / 2 / 4</f>
+        <f t="shared" si="8"/>
         <v>1.2500000000000002E-7</v>
       </c>
     </row>
@@ -3295,55 +3294,55 @@
         <v>0.10886399999999999</v>
       </c>
       <c r="H22" s="10">
-        <f t="shared" ref="H22:T22" si="5">0.84*(0.36^2)</f>
+        <f t="shared" ref="H22:T22" si="9">0.84*(0.36^2)</f>
         <v>0.10886399999999999</v>
       </c>
       <c r="I22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="J22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="K22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="L22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="M22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="N22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="O22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="P22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="Q22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="R22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="S22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
       <c r="T22" s="10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v>0.10886399999999999</v>
       </c>
     </row>
@@ -3495,55 +3494,55 @@
         <v>0.2</v>
       </c>
       <c r="H25" s="10">
-        <f t="shared" ref="H25:T25" si="6">2*0.1</f>
+        <f t="shared" ref="H25:T25" si="10">2*0.1</f>
         <v>0.2</v>
       </c>
       <c r="I25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="J25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="K25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="L25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="M25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="N25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="O25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="P25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="Q25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="R25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="S25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
       <c r="T25" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0.2</v>
       </c>
     </row>
@@ -3632,55 +3631,55 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="H27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" ref="H27:T27" si="11">0.00001 /2</f>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="I27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="J27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="K27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="L27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="M27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="N27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="O27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="P27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="Q27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="R27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="S27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="T27" s="10">
-        <f>0.00001 /2</f>
+        <f t="shared" si="11"/>
         <v>5.0000000000000004E-6</v>
       </c>
     </row>
@@ -3707,55 +3706,55 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="H28" s="10">
-        <f t="shared" ref="H28:T28" si="7">0.000000005 / 5</f>
+        <f t="shared" ref="H28:T28" si="12">0.000000005 / 5</f>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="I28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="J28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="K28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="L28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="M28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="N28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="O28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="P28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="Q28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="R28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="S28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="T28" s="10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0000000000000001E-9</v>
       </c>
     </row>
@@ -3779,7 +3778,7 @@
         <v>239</v>
       </c>
       <c r="G29" s="10">
-        <f t="shared" ref="G29" si="8">0.00002 / 14 / 5</f>
+        <f t="shared" ref="G29" si="13">0.00002 / 14 / 5</f>
         <v>2.8571428571428575E-7</v>
       </c>
       <c r="H29" s="10">
@@ -3842,7 +3841,7 @@
         <v>239</v>
       </c>
       <c r="G30" s="10">
-        <f t="shared" ref="G30" si="9">0.00002 / 14 / 5 /10</f>
+        <f t="shared" ref="G30" si="14">0.00002 / 14 / 5 /10</f>
         <v>2.8571428571428575E-8</v>
       </c>
       <c r="H30" s="10">
@@ -3908,8 +3907,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21:T21">
-    <cfRule type="colorScale" priority="596">
+  <conditionalFormatting sqref="G30:T30">
+    <cfRule type="colorScale" priority="601">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3919,51 +3918,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="597">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29:T30">
-    <cfRule type="colorScale" priority="598">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="599">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G30:T30">
     <cfRule type="colorScale" priority="600">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="601">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3975,7 +3930,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:T6">
-    <cfRule type="colorScale" priority="603">
+    <cfRule type="colorScale" priority="604">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3985,7 +3940,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="604">
+    <cfRule type="colorScale" priority="603">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4019,7 +3974,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8:T8">
-    <cfRule type="colorScale" priority="607">
+    <cfRule type="colorScale" priority="608">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4029,7 +3984,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="608">
+    <cfRule type="colorScale" priority="607">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4041,7 +3996,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:T9">
-    <cfRule type="colorScale" priority="609">
+    <cfRule type="colorScale" priority="610">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4051,7 +4006,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="610">
+    <cfRule type="colorScale" priority="609">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4063,7 +4018,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:T10">
-    <cfRule type="colorScale" priority="611">
+    <cfRule type="colorScale" priority="612">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4073,7 +4028,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="612">
+    <cfRule type="colorScale" priority="611">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4085,7 +4040,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:T11">
-    <cfRule type="colorScale" priority="613">
+    <cfRule type="colorScale" priority="614">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4095,7 +4050,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="614">
+    <cfRule type="colorScale" priority="613">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4107,7 +4062,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14:T14">
-    <cfRule type="colorScale" priority="615">
+    <cfRule type="colorScale" priority="616">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4117,7 +4072,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="616">
+    <cfRule type="colorScale" priority="615">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4129,7 +4084,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15:T17">
-    <cfRule type="colorScale" priority="617">
+    <cfRule type="colorScale" priority="618">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4139,7 +4094,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="618">
+    <cfRule type="colorScale" priority="617">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4151,16 +4106,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H18:T18">
-    <cfRule type="colorScale" priority="619">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="620">
       <colorScale>
         <cfvo type="min"/>
@@ -4171,41 +4116,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H22:T22">
-    <cfRule type="colorScale" priority="621">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="622">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H23:T28">
-    <cfRule type="colorScale" priority="623">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="624">
+    <cfRule type="colorScale" priority="619">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4238,8 +4149,84 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3">
-    <cfRule type="colorScale" priority="25">
+  <conditionalFormatting sqref="H21:T21">
+    <cfRule type="colorScale" priority="596">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="597">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H22:T22">
+    <cfRule type="colorScale" priority="622">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="621">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23:T28">
+    <cfRule type="colorScale" priority="624">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="623">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29:T30">
+    <cfRule type="colorScale" priority="598">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="599">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4261,6 +4248,16 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3">
     <cfRule type="colorScale" priority="23">
@@ -4273,21 +4270,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3">
     <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3">
-    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4309,9 +4292,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L3">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4333,9 +4314,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M3">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4357,9 +4336,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N3">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4381,9 +4358,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O3">
-    <cfRule type="colorScale" priority="13">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4405,9 +4380,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P3">
-    <cfRule type="colorScale" priority="11">
+    <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4429,6 +4402,16 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q3">
     <cfRule type="colorScale" priority="9">
@@ -4441,21 +4424,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q3">
     <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R3">
-    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4477,9 +4446,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S3">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4501,6 +4468,16 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T3">
     <cfRule type="colorScale" priority="1">
@@ -4513,8 +4490,6 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T3">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
ongoing rc debug since wb
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_25_07_02.xlsx
+++ b/simulations/scene/inputs/Scenarios_25_07_02.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp04472\home\torisuten\package\Root-CyNAPS\simulations\scene\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp20259\work_home\tigerault\Wheat-BRIDGES_framework\Root-CyNAPS\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F01D3E4-8ADE-46F4-AA05-664C7AD0C1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BEF7B1-06F4-438A-8D2F-3FD9FCA17DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="285">
   <si>
     <t>input_file</t>
   </si>
@@ -883,6 +883,12 @@
   </si>
   <si>
     <t>root02494.pckl</t>
+  </si>
+  <si>
+    <t>Cv_AA_phloem_collar</t>
+  </si>
+  <si>
+    <t>Enforced amino acids volumic concentration at the shoot-root junction</t>
   </si>
 </sst>
 </file>
@@ -1812,7 +1818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.7109375" style="1" customWidth="1"/>
@@ -3872,6 +3878,68 @@
         <v>0</v>
       </c>
     </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="G31" s="14">
+        <v>260</v>
+      </c>
+      <c r="H31" s="1">
+        <v>260</v>
+      </c>
+      <c r="I31" s="1">
+        <v>260</v>
+      </c>
+      <c r="J31" s="1">
+        <v>260</v>
+      </c>
+      <c r="K31" s="1">
+        <v>260</v>
+      </c>
+      <c r="L31" s="1">
+        <v>260</v>
+      </c>
+      <c r="M31" s="1">
+        <v>260</v>
+      </c>
+      <c r="N31" s="1">
+        <v>260</v>
+      </c>
+      <c r="O31" s="1">
+        <v>260</v>
+      </c>
+      <c r="P31" s="1">
+        <v>260</v>
+      </c>
+      <c r="Q31" s="1">
+        <v>260</v>
+      </c>
+      <c r="R31" s="1">
+        <v>260</v>
+      </c>
+      <c r="S31" s="1">
+        <v>260</v>
+      </c>
+      <c r="T31" s="1">
+        <v>260</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="G29:G30">
     <cfRule type="colorScale" priority="593">
@@ -4775,6 +4843,28 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q16:T16">
+    <cfRule type="colorScale" priority="72">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="71">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="Q17:T17 Q15:T15">
     <cfRule type="colorScale" priority="93">
       <colorScale>
@@ -4787,28 +4877,6 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="94">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q16:T16">
-    <cfRule type="colorScale" priority="72">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="71">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>